<commit_message>
Edited station depth flags
</commit_message>
<xml_diff>
--- a/Meta/flagsMap_withDecisions.xlsx
+++ b/Meta/flagsMap_withDecisions.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/vitense_kelsey_epa_gov/Documents/GL_Data/Meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="649" documentId="13_ncr:4000b_{6437034B-B068-4CF2-9A04-9208A97A6BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{796D601A-E972-4E5B-BD96-5B079AEAE3FB}"/>
+  <xr:revisionPtr revIDLastSave="663" documentId="13_ncr:4000b_{6437034B-B068-4CF2-9A04-9208A97A6BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7B067EB-D55D-4915-8E3D-AEB601511FD3}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="19440" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-61548" yWindow="-1872" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="flagsMap_withDecisions" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">flagsMap_withDecisions!$A$1:$A$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">flagsMap_withDecisions!$A$1:$A$107</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -97,7 +97,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="188">
   <si>
     <t>Study</t>
   </si>
@@ -630,21 +630,9 @@
     <t>D</t>
   </si>
   <si>
-    <t>Station depth imputed</t>
-  </si>
-  <si>
-    <t>Station depth imputed from another site visit</t>
-  </si>
-  <si>
-    <t>Station depth imputed from maximum CTD sample depth</t>
-  </si>
-  <si>
     <t>SeaBird</t>
   </si>
   <si>
-    <t>NOAActd</t>
-  </si>
-  <si>
     <t>No result recorded.</t>
   </si>
   <si>
@@ -667,6 +655,12 @@
   </si>
   <si>
     <t>We don't know what this is and already removed anyway.</t>
+  </si>
+  <si>
+    <t>Station depth estimated as max CTD sample depth</t>
+  </si>
+  <si>
+    <t>station Depth estimated as the maximum CTD Depth</t>
   </si>
 </sst>
 </file>
@@ -1641,21 +1635,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T113"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:T110"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5546875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="44.33203125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="38.5546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="44.28515625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="38.5703125" style="1" customWidth="1"/>
     <col min="5" max="5" width="15" style="6" customWidth="1"/>
     <col min="6" max="6" width="26" style="6" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" style="6" customWidth="1"/>
-    <col min="8" max="8" width="35.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="6"/>
+    <col min="7" max="7" width="10.5703125" style="6" customWidth="1"/>
+    <col min="8" max="8" width="35.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1681,7 +1675,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>171</v>
       </c>
@@ -1707,7 +1701,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>86</v>
       </c>
@@ -1733,7 +1727,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>52</v>
       </c>
@@ -1759,7 +1753,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>50</v>
       </c>
@@ -1785,7 +1779,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>29</v>
       </c>
@@ -1811,7 +1805,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>170</v>
       </c>
@@ -1837,7 +1831,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>171</v>
       </c>
@@ -1863,7 +1857,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>86</v>
       </c>
@@ -1889,7 +1883,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>52</v>
       </c>
@@ -1915,7 +1909,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>50</v>
       </c>
@@ -1941,7 +1935,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>29</v>
       </c>
@@ -1967,7 +1961,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>170</v>
       </c>
@@ -1993,7 +1987,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>171</v>
       </c>
@@ -2016,7 +2010,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>86</v>
       </c>
@@ -2039,7 +2033,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>52</v>
       </c>
@@ -2062,7 +2056,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>50</v>
       </c>
@@ -2085,7 +2079,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>29</v>
       </c>
@@ -2108,7 +2102,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>170</v>
       </c>
@@ -2131,7 +2125,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>4</v>
       </c>
@@ -2149,7 +2143,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>4</v>
       </c>
@@ -2170,7 +2164,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>4</v>
       </c>
@@ -2193,7 +2187,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>4</v>
       </c>
@@ -2219,7 +2213,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>4</v>
       </c>
@@ -2239,7 +2233,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>4</v>
       </c>
@@ -2259,7 +2253,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>4</v>
       </c>
@@ -2277,7 +2271,7 @@
       </c>
       <c r="H26" s="7"/>
     </row>
-    <row r="27" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>4</v>
       </c>
@@ -2295,7 +2289,7 @@
       </c>
       <c r="H27" s="7"/>
     </row>
-    <row r="28" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>4</v>
       </c>
@@ -2313,7 +2307,7 @@
       </c>
       <c r="H28" s="7"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>4</v>
       </c>
@@ -2328,7 +2322,7 @@
       </c>
       <c r="H29" s="11"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>4</v>
       </c>
@@ -2343,7 +2337,7 @@
       </c>
       <c r="H30" s="11"/>
     </row>
-    <row r="31" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>4</v>
       </c>
@@ -2360,7 +2354,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>4</v>
       </c>
@@ -2377,7 +2371,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>4</v>
       </c>
@@ -2394,7 +2388,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>4</v>
       </c>
@@ -2411,7 +2405,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>4</v>
       </c>
@@ -2431,7 +2425,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
         <v>4</v>
       </c>
@@ -2454,7 +2448,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
         <v>4</v>
       </c>
@@ -2477,7 +2471,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>23</v>
       </c>
@@ -2491,7 +2485,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>23</v>
       </c>
@@ -2505,7 +2499,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>23</v>
       </c>
@@ -2531,7 +2525,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>27</v>
       </c>
@@ -2557,7 +2551,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>27</v>
       </c>
@@ -2580,7 +2574,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>29</v>
       </c>
@@ -2606,7 +2600,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>29</v>
       </c>
@@ -2630,7 +2624,7 @@
       </c>
       <c r="H44" s="7"/>
     </row>
-    <row r="45" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>29</v>
       </c>
@@ -2651,7 +2645,7 @@
       </c>
       <c r="H45" s="7"/>
     </row>
-    <row r="46" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>29</v>
       </c>
@@ -2677,7 +2671,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>29</v>
       </c>
@@ -2700,7 +2694,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>29</v>
       </c>
@@ -2720,7 +2714,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>29</v>
       </c>
@@ -2743,7 +2737,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>29</v>
       </c>
@@ -2763,7 +2757,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="51" spans="1:20" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>29</v>
       </c>
@@ -2777,7 +2771,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>29</v>
       </c>
@@ -2797,7 +2791,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>29</v>
       </c>
@@ -2814,7 +2808,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="54" spans="1:20" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>29</v>
       </c>
@@ -2834,7 +2828,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="55" spans="1:20" s="7" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:20" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
         <v>50</v>
       </c>
@@ -2858,7 +2852,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="56" spans="1:20" s="10" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:20" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
         <v>50</v>
       </c>
@@ -2894,7 +2888,7 @@
       <c r="S56" s="7"/>
       <c r="T56" s="7"/>
     </row>
-    <row r="57" spans="1:20" s="10" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:20" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
         <v>50</v>
       </c>
@@ -2928,7 +2922,7 @@
       <c r="S57" s="7"/>
       <c r="T57" s="7"/>
     </row>
-    <row r="58" spans="1:20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>50</v>
       </c>
@@ -2951,7 +2945,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="59" spans="1:20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>50</v>
       </c>
@@ -2974,7 +2968,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="60" spans="1:20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>50</v>
       </c>
@@ -2997,7 +2991,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="61" spans="1:20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>50</v>
       </c>
@@ -3020,7 +3014,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="62" spans="1:20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>50</v>
       </c>
@@ -3043,7 +3037,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="63" spans="1:20" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:20" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>50</v>
       </c>
@@ -3077,7 +3071,7 @@
       <c r="S63" s="7"/>
       <c r="T63" s="7"/>
     </row>
-    <row r="64" spans="1:20" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:20" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>50</v>
       </c>
@@ -3111,7 +3105,7 @@
       <c r="S64" s="7"/>
       <c r="T64" s="7"/>
     </row>
-    <row r="65" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" ht="45.75" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>52</v>
       </c>
@@ -3135,7 +3129,7 @@
       </c>
       <c r="H65" s="7"/>
     </row>
-    <row r="66" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>52</v>
       </c>
@@ -3158,7 +3152,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>52</v>
       </c>
@@ -3181,7 +3175,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>52</v>
       </c>
@@ -3204,7 +3198,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>52</v>
       </c>
@@ -3227,7 +3221,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>52</v>
       </c>
@@ -3253,7 +3247,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>52</v>
       </c>
@@ -3276,7 +3270,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>52</v>
       </c>
@@ -3299,7 +3293,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="21.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>52</v>
       </c>
@@ -3322,7 +3316,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>52</v>
       </c>
@@ -3348,7 +3342,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>52</v>
       </c>
@@ -3371,7 +3365,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>52</v>
       </c>
@@ -3394,7 +3388,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="21.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>52</v>
       </c>
@@ -3417,7 +3411,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>52</v>
       </c>
@@ -3440,7 +3434,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>52</v>
       </c>
@@ -3463,7 +3457,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="21.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>52</v>
       </c>
@@ -3480,7 +3474,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="21.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
         <v>52</v>
       </c>
@@ -3503,7 +3497,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" ht="45.75" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>52</v>
       </c>
@@ -3529,7 +3523,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="52.2" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" ht="57" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
         <v>52</v>
       </c>
@@ -3552,7 +3546,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
         <v>52</v>
       </c>
@@ -3575,7 +3569,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
         <v>52</v>
       </c>
@@ -3592,7 +3586,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="42" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" ht="57" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
         <v>52</v>
       </c>
@@ -3615,7 +3609,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
         <v>52</v>
       </c>
@@ -3638,7 +3632,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
         <v>52</v>
       </c>
@@ -3664,7 +3658,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
         <v>52</v>
       </c>
@@ -3687,7 +3681,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A90" s="6" t="s">
         <v>52</v>
       </c>
@@ -3710,7 +3704,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
         <v>52</v>
       </c>
@@ -3733,7 +3727,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A92" s="6" t="s">
         <v>52</v>
       </c>
@@ -3752,7 +3746,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
         <v>52</v>
       </c>
@@ -3760,7 +3754,7 @@
         <v>53</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D93" s="3"/>
       <c r="E93" s="7"/>
@@ -3769,7 +3763,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="6" t="s">
         <v>52</v>
       </c>
@@ -3777,7 +3771,7 @@
         <v>53</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D94" s="3"/>
       <c r="E94" s="7"/>
@@ -3786,7 +3780,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
         <v>52</v>
       </c>
@@ -3794,7 +3788,7 @@
         <v>53</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D95" s="3"/>
       <c r="E95" s="7"/>
@@ -3803,7 +3797,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
         <v>52</v>
       </c>
@@ -3811,7 +3805,7 @@
         <v>53</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D96" s="3"/>
       <c r="E96" s="7"/>
@@ -3820,7 +3814,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="21.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A97" s="6" t="s">
         <v>52</v>
       </c>
@@ -3843,7 +3837,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
         <v>52</v>
       </c>
@@ -3860,7 +3854,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="42" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" ht="45.75" x14ac:dyDescent="0.25">
       <c r="A99" s="6" t="s">
         <v>52</v>
       </c>
@@ -3883,7 +3877,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
         <v>52</v>
       </c>
@@ -3900,7 +3894,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
         <v>52</v>
       </c>
@@ -3915,7 +3909,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A102" s="6" t="s">
         <v>52</v>
       </c>
@@ -3938,7 +3932,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="103" spans="1:8" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" s="7" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A103" s="7" t="s">
         <v>86</v>
       </c>
@@ -3962,7 +3956,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="104" spans="1:8" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" s="7" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A104" s="7" t="s">
         <v>171</v>
       </c>
@@ -3986,7 +3980,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" s="6" t="s">
         <v>170</v>
       </c>
@@ -4010,141 +4004,81 @@
         <v>152</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A106" s="6" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B106" s="6" t="s">
         <v>176</v>
       </c>
       <c r="C106" s="6" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>176</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="G106" s="14" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A107" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="B107" s="6" t="s">
-        <v>176</v>
+        <v>52</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="E107" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="F107" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="G107" s="14" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
+        <v>181</v>
+      </c>
+      <c r="D107" s="2"/>
+      <c r="G107" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H107" s="7" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A108" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B108" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C108" s="6" t="s">
-        <v>178</v>
-      </c>
+      <c r="C108" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="D108" s="2"/>
       <c r="E108" s="6" t="s">
         <v>176</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="G108" s="14" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="109" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A109" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="B109" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="C109" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="E109" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="F109" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="G109" s="14" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="110" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A110" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C110" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="D110" s="2"/>
-      <c r="G110" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="H110" s="7" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A111" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="B111" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C111" s="18" t="s">
-        <v>187</v>
-      </c>
-      <c r="D111" s="2"/>
-      <c r="E111" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="F111" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="G111" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="H111" s="7"/>
-    </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A112" s="7"/>
-      <c r="B112" s="7"/>
-      <c r="C112" s="7"/>
-      <c r="D112"/>
-      <c r="G112" s="19"/>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A113" s="7"/>
-      <c r="B113"/>
-      <c r="C113" s="17" t="s">
-        <v>187</v>
-      </c>
-      <c r="D113"/>
-      <c r="G113" s="19"/>
+      <c r="H108" s="7"/>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109" s="7"/>
+      <c r="B109" s="7"/>
+      <c r="C109" s="7"/>
+      <c r="D109"/>
+      <c r="G109" s="19"/>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110" s="7"/>
+      <c r="B110"/>
+      <c r="C110" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="D110"/>
+      <c r="G110" s="19"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A110" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:A107" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
@@ -4161,12 +4095,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100919AB8A12910594B8F4D80F4ACA7D0E7" ma:contentTypeVersion="6" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9c71394a73500791d9f4b659570ff6f6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a318c9bd-5828-4914-8ac9-a57d8c01df7a" xmlns:ns3="4da7f078-0f32-436f-b12a-21525bae5a0e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f0993cb8e7f28d1e7915cb051b812a71" ns2:_="" ns3:_="">
     <xsd:import namespace="a318c9bd-5828-4914-8ac9-a57d8c01df7a"/>
@@ -4343,6 +4271,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B8261F5-E2C2-49F8-99F3-13EB69507EB7}">
   <ds:schemaRefs>
@@ -4352,15 +4286,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC4DE233-B05C-40D4-9E0D-B697BD35B3E3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56F0D49C-4924-48A7-977F-FB48DDC11B03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4377,4 +4302,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC4DE233-B05C-40D4-9E0D-B697BD35B3E3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Edited flagsMap to remove any remaining observations with no measurement or depth greater than station depth flag in NCCA 2015 hydro
</commit_message>
<xml_diff>
--- a/Meta/flagsMap_withDecisions.xlsx
+++ b/Meta/flagsMap_withDecisions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/vitense_kelsey_epa_gov/Documents/GL_Data/Meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="663" documentId="13_ncr:4000b_{6437034B-B068-4CF2-9A04-9208A97A6BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7B067EB-D55D-4915-8E3D-AEB601511FD3}"/>
+  <xr:revisionPtr revIDLastSave="672" documentId="13_ncr:4000b_{6437034B-B068-4CF2-9A04-9208A97A6BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C77D7675-8E72-4084-8362-12EB2C508CA2}"/>
   <bookViews>
-    <workbookView xWindow="-61548" yWindow="-1872" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="19440" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="flagsMap_withDecisions" sheetId="1" r:id="rId1"/>
@@ -603,12 +603,6 @@
     <t>below MDL</t>
   </si>
   <si>
-    <t>Should be removed anyway because all NA</t>
-  </si>
-  <si>
-    <t>only catches one case of where UW &gt; AMB light. There are other similar cases as well, so don't remove these.</t>
-  </si>
-  <si>
     <t>NOAA_WQ</t>
   </si>
   <si>
@@ -661,6 +655,12 @@
   </si>
   <si>
     <t>station Depth estimated as the maximum CTD Depth</t>
+  </si>
+  <si>
+    <t>Will be removed for most anyway because RESULT is NA, or is mapped to Remove in Analytes3</t>
+  </si>
+  <si>
+    <t>Only catches one case of where UW &gt; AMB light. There are other similar cases as well, so don't remove these (and this comment is applied to  analytes other than CPAR at same depth). Add flag in joined dataset for CPAR&gt;100%</t>
   </si>
 </sst>
 </file>
@@ -1636,20 +1636,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T110"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="44.28515625" style="6" customWidth="1"/>
-    <col min="4" max="4" width="38.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="44.33203125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="38.5546875" style="1" customWidth="1"/>
     <col min="5" max="5" width="15" style="6" customWidth="1"/>
     <col min="6" max="6" width="26" style="6" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="35.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.85546875" style="6"/>
+    <col min="7" max="7" width="10.5546875" style="6" customWidth="1"/>
+    <col min="8" max="8" width="35.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1675,9 +1675,9 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>166</v>
@@ -1701,7 +1701,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>86</v>
       </c>
@@ -1727,7 +1727,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>52</v>
       </c>
@@ -1753,7 +1753,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>50</v>
       </c>
@@ -1779,7 +1779,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>29</v>
       </c>
@@ -1805,9 +1805,9 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>166</v>
@@ -1831,18 +1831,18 @@
         <v>138</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>173</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>15</v>
@@ -1854,21 +1854,21 @@
         <v>132</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>86</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>15</v>
@@ -1880,21 +1880,21 @@
         <v>132</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>52</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>15</v>
@@ -1906,21 +1906,21 @@
         <v>132</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>50</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>15</v>
@@ -1932,21 +1932,21 @@
         <v>132</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>29</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>15</v>
@@ -1958,21 +1958,21 @@
         <v>132</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>172</v>
-      </c>
       <c r="C13" s="6" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>15</v>
@@ -1984,12 +1984,12 @@
         <v>132</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>128</v>
@@ -1998,7 +1998,7 @@
         <v>128</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>94</v>
@@ -2010,7 +2010,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>86</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>128</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>94</v>
@@ -2033,7 +2033,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>52</v>
       </c>
@@ -2044,7 +2044,7 @@
         <v>128</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>94</v>
@@ -2056,7 +2056,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>50</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>128</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>94</v>
@@ -2079,7 +2079,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>29</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>128</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>94</v>
@@ -2102,9 +2102,9 @@
         <v>89</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>128</v>
@@ -2113,7 +2113,7 @@
         <v>128</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>94</v>
@@ -2125,7 +2125,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>4</v>
       </c>
@@ -2143,7 +2143,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>4</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>4</v>
       </c>
@@ -2187,7 +2187,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>4</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>4</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>4</v>
       </c>
@@ -2253,7 +2253,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>4</v>
       </c>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="H26" s="7"/>
     </row>
-    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>4</v>
       </c>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="H27" s="7"/>
     </row>
-    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>4</v>
       </c>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="H28" s="7"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>4</v>
       </c>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="H29" s="11"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>4</v>
       </c>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="H30" s="11"/>
     </row>
-    <row r="31" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>4</v>
       </c>
@@ -2354,7 +2354,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
         <v>4</v>
       </c>
@@ -2371,7 +2371,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>4</v>
       </c>
@@ -2388,7 +2388,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>4</v>
       </c>
@@ -2405,7 +2405,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>4</v>
       </c>
@@ -2425,7 +2425,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
         <v>4</v>
       </c>
@@ -2448,7 +2448,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
         <v>4</v>
       </c>
@@ -2471,21 +2471,21 @@
         <v>89</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G38" s="16" t="s">
-        <v>89</v>
+      <c r="G38" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>23</v>
       </c>
@@ -2496,10 +2496,10 @@
         <v>89</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
         <v>23</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>27</v>
       </c>
@@ -2551,7 +2551,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>27</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>29</v>
       </c>
@@ -2600,7 +2600,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>29</v>
       </c>
@@ -2624,7 +2624,7 @@
       </c>
       <c r="H44" s="7"/>
     </row>
-    <row r="45" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>29</v>
       </c>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="H45" s="7"/>
     </row>
-    <row r="46" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>29</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>29</v>
       </c>
@@ -2694,7 +2694,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>29</v>
       </c>
@@ -2714,7 +2714,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="49" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>29</v>
       </c>
@@ -2737,7 +2737,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="50" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
         <v>29</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="51" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:20" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
         <v>29</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="52" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
         <v>29</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="53" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
         <v>29</v>
       </c>
@@ -2808,7 +2808,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="54" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:20" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
         <v>29</v>
       </c>
@@ -2828,7 +2828,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="55" spans="1:20" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:20" s="7" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A55" s="10" t="s">
         <v>50</v>
       </c>
@@ -2852,7 +2852,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="56" spans="1:20" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:20" s="10" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
         <v>50</v>
       </c>
@@ -2888,7 +2888,7 @@
       <c r="S56" s="7"/>
       <c r="T56" s="7"/>
     </row>
-    <row r="57" spans="1:20" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:20" s="10" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A57" s="7" t="s">
         <v>50</v>
       </c>
@@ -2922,7 +2922,7 @@
       <c r="S57" s="7"/>
       <c r="T57" s="7"/>
     </row>
-    <row r="58" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:20" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>50</v>
       </c>
@@ -2945,7 +2945,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="59" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:20" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>50</v>
       </c>
@@ -2968,7 +2968,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="60" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:20" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>50</v>
       </c>
@@ -2991,7 +2991,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="61" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:20" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>50</v>
       </c>
@@ -3014,7 +3014,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="62" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:20" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>50</v>
       </c>
@@ -3037,7 +3037,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="63" spans="1:20" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:20" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A63" s="7" t="s">
         <v>50</v>
       </c>
@@ -3071,7 +3071,7 @@
       <c r="S63" s="7"/>
       <c r="T63" s="7"/>
     </row>
-    <row r="64" spans="1:20" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:20" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A64" s="7" t="s">
         <v>50</v>
       </c>
@@ -3105,7 +3105,7 @@
       <c r="S64" s="7"/>
       <c r="T64" s="7"/>
     </row>
-    <row r="65" spans="1:8" ht="45.75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>52</v>
       </c>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="H65" s="7"/>
     </row>
-    <row r="66" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
         <v>52</v>
       </c>
@@ -3152,7 +3152,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
         <v>52</v>
       </c>
@@ -3175,7 +3175,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A68" s="6" t="s">
         <v>52</v>
       </c>
@@ -3198,7 +3198,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
         <v>52</v>
       </c>
@@ -3221,7 +3221,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="165" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
         <v>52</v>
       </c>
@@ -3247,7 +3247,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
         <v>52</v>
       </c>
@@ -3270,7 +3270,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A72" s="6" t="s">
         <v>52</v>
       </c>
@@ -3293,7 +3293,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A73" s="6" t="s">
         <v>52</v>
       </c>
@@ -3316,7 +3316,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
         <v>52</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
         <v>52</v>
       </c>
@@ -3365,7 +3365,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A76" s="6" t="s">
         <v>52</v>
       </c>
@@ -3388,7 +3388,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
         <v>52</v>
       </c>
@@ -3411,7 +3411,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A78" s="6" t="s">
         <v>52</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
         <v>52</v>
       </c>
@@ -3457,7 +3457,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
         <v>52</v>
       </c>
@@ -3474,7 +3474,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A81" s="6" t="s">
         <v>52</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="45.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
         <v>52</v>
       </c>
@@ -3523,7 +3523,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="57" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" ht="52.2" x14ac:dyDescent="0.3">
       <c r="A83" s="6" t="s">
         <v>52</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
         <v>52</v>
       </c>
@@ -3569,7 +3569,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="85" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A85" s="6" t="s">
         <v>52</v>
       </c>
@@ -3586,7 +3586,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="57" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" ht="42" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
         <v>52</v>
       </c>
@@ -3609,7 +3609,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A87" s="6" t="s">
         <v>52</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A88" s="6" t="s">
         <v>52</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
         <v>52</v>
       </c>
@@ -3681,7 +3681,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A90" s="6" t="s">
         <v>52</v>
       </c>
@@ -3704,7 +3704,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A91" s="6" t="s">
         <v>52</v>
       </c>
@@ -3727,7 +3727,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A92" s="6" t="s">
         <v>52</v>
       </c>
@@ -3746,7 +3746,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" s="6" t="s">
         <v>52</v>
       </c>
@@ -3754,7 +3754,7 @@
         <v>53</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D93" s="3"/>
       <c r="E93" s="7"/>
@@ -3763,7 +3763,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
         <v>52</v>
       </c>
@@ -3771,7 +3771,7 @@
         <v>53</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D94" s="3"/>
       <c r="E94" s="7"/>
@@ -3780,7 +3780,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" s="6" t="s">
         <v>52</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>53</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D95" s="3"/>
       <c r="E95" s="7"/>
@@ -3797,7 +3797,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" s="6" t="s">
         <v>52</v>
       </c>
@@ -3805,7 +3805,7 @@
         <v>53</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D96" s="3"/>
       <c r="E96" s="7"/>
@@ -3814,7 +3814,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" ht="21.6" x14ac:dyDescent="0.3">
       <c r="A97" s="6" t="s">
         <v>52</v>
       </c>
@@ -3837,7 +3837,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A98" s="6" t="s">
         <v>52</v>
       </c>
@@ -3854,7 +3854,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="45.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" ht="42" x14ac:dyDescent="0.3">
       <c r="A99" s="6" t="s">
         <v>52</v>
       </c>
@@ -3877,7 +3877,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="100" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" s="6" t="s">
         <v>52</v>
       </c>
@@ -3894,7 +3894,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="6" t="s">
         <v>52</v>
       </c>
@@ -3909,7 +3909,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" ht="31.8" x14ac:dyDescent="0.3">
       <c r="A102" s="6" t="s">
         <v>52</v>
       </c>
@@ -3932,7 +3932,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="103" spans="1:8" s="7" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A103" s="7" t="s">
         <v>86</v>
       </c>
@@ -3956,9 +3956,9 @@
         <v>138</v>
       </c>
     </row>
-    <row r="104" spans="1:8" s="7" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" s="7" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A104" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B104" s="7" t="s">
         <v>53</v>
@@ -3980,9 +3980,9 @@
         <v>138</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B105" s="6" t="s">
         <v>28</v>
@@ -4004,75 +4004,75 @@
         <v>152</v>
       </c>
     </row>
-    <row r="106" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A106" s="6" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C106" s="6" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G106" s="14" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A107" s="6" t="s">
         <v>52</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D107" s="2"/>
       <c r="G107" s="15" t="s">
         <v>25</v>
       </c>
       <c r="H107" s="7" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A108" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="B108" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="C108" s="18" t="s">
         <v>185</v>
-      </c>
-    </row>
-    <row r="108" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A108" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="B108" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="C108" s="18" t="s">
-        <v>187</v>
       </c>
       <c r="D108" s="2"/>
       <c r="E108" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G108" s="14" t="s">
         <v>89</v>
       </c>
       <c r="H108" s="7"/>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" s="7"/>
       <c r="B109" s="7"/>
       <c r="C109" s="7"/>
       <c r="D109"/>
       <c r="G109" s="19"/>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" s="7"/>
       <c r="B110"/>
       <c r="C110" s="17" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D110"/>
       <c r="G110" s="19"/>
@@ -4086,15 +4086,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100919AB8A12910594B8F4D80F4ACA7D0E7" ma:contentTypeVersion="6" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9c71394a73500791d9f4b659570ff6f6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a318c9bd-5828-4914-8ac9-a57d8c01df7a" xmlns:ns3="4da7f078-0f32-436f-b12a-21525bae5a0e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f0993cb8e7f28d1e7915cb051b812a71" ns2:_="" ns3:_="">
     <xsd:import namespace="a318c9bd-5828-4914-8ac9-a57d8c01df7a"/>
@@ -4271,6 +4262,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -4278,14 +4278,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B8261F5-E2C2-49F8-99F3-13EB69507EB7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56F0D49C-4924-48A7-977F-FB48DDC11B03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4304,6 +4296,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B8261F5-E2C2-49F8-99F3-13EB69507EB7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC4DE233-B05C-40D4-9E0D-B697BD35B3E3}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Removed QAcomment for NCCA water chem 2010 because not in data
</commit_message>
<xml_diff>
--- a/Meta/flagsMap_withDecisions.xlsx
+++ b/Meta/flagsMap_withDecisions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/vitense_kelsey_epa_gov/Documents/GL_Data/Meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="703" documentId="13_ncr:4000b_{6437034B-B068-4CF2-9A04-9208A97A6BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62B076F7-0EA1-4EAF-87DE-4D3FC3BD5722}"/>
+  <xr:revisionPtr revIDLastSave="715" documentId="13_ncr:4000b_{6437034B-B068-4CF2-9A04-9208A97A6BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{621A1976-AB3A-4FC8-ABBC-CDCB878B0B22}"/>
   <bookViews>
     <workbookView xWindow="-61548" yWindow="-1872" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="flagsMap_withDecisions" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">flagsMap_withDecisions!$A$1:$A$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">flagsMap_withDecisions!$A$1:$A$100</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
@@ -29,7 +29,6 @@
     <author>tc={9DD5E251-9F0E-49B4-8118-B96699C3281D}</author>
     <author>tc={57535352-09AF-42AB-BEBD-584FAEC623BD}</author>
     <author>tc={A8BE5C20-40BD-42DF-838C-01B7D5AFF883}</author>
-    <author>tc={6A749074-B681-48EE-9D60-AAD094A450F9}</author>
   </authors>
   <commentList>
     <comment ref="E1" authorId="0" shapeId="0" xr:uid="{068A9404-2F3B-466F-9954-2FBC3269B52F}">
@@ -74,20 +73,12 @@
     In current flagsMap.csv, did not include R-no reported units because should go with U (row 47). Did not include Q10,R-recorded mean secchi depth is greater than station depth because it's for NC, not GL.</t>
       </text>
     </comment>
-    <comment ref="A40" authorId="4" shapeId="0" xr:uid="{6A749074-B681-48EE-9D60-AAD094A450F9}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Note: Did not include 3 extra flags in current flagsMap.csv here with repeat QAcomment in QAcode</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="185">
   <si>
     <t>Study</t>
   </si>
@@ -1592,15 +1583,12 @@
   <threadedComment ref="A20" dT="2024-08-14T17:33:35.12" personId="{661D028C-1F83-4763-B7EC-DB616DE23CF1}" id="{A8BE5C20-40BD-42DF-838C-01B7D5AFF883}">
     <text>In current flagsMap.csv, did not include R-no reported units because should go with U (row 47). Did not include Q10,R-recorded mean secchi depth is greater than station depth because it's for NC, not GL.</text>
   </threadedComment>
-  <threadedComment ref="A40" dT="2024-08-14T17:05:26.53" personId="{661D028C-1F83-4763-B7EC-DB616DE23CF1}" id="{6A749074-B681-48EE-9D60-AAD094A450F9}">
-    <text>Note: Did not include 3 extra flags in current flagsMap.csv here with repeat QAcomment in QAcode</text>
-  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T109"/>
+  <dimension ref="A1:T106"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" style="6" bestFit="1" customWidth="1"/>
@@ -2468,9 +2456,6 @@
       <c r="B40" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C40" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="D40" s="1" t="s">
         <v>29</v>
       </c>
@@ -2494,9 +2479,6 @@
       <c r="B41" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C41" s="6" t="s">
-        <v>31</v>
-      </c>
       <c r="D41" s="1" t="s">
         <v>31</v>
       </c>
@@ -2511,51 +2493,47 @@
       </c>
       <c r="H41" s="7"/>
     </row>
-    <row r="42" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="G42" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="H42" s="7"/>
-    </row>
-    <row r="43" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="G42" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="G43" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="H43" s="6" t="s">
-        <v>134</v>
+        <v>126</v>
+      </c>
+      <c r="G43" s="14" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2563,19 +2541,16 @@
         <v>27</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E44" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>126</v>
+        <v>36</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>115</v>
       </c>
       <c r="G44" s="14" t="s">
         <v>87</v>
@@ -2586,16 +2561,16 @@
         <v>27</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="F45" s="6" t="s">
-        <v>115</v>
+        <v>90</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="G45" s="14" t="s">
         <v>87</v>
@@ -2606,22 +2581,13 @@
         <v>27</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F46" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G46" s="14" t="s">
-        <v>87</v>
+        <v>42</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="G46" s="15" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2629,19 +2595,16 @@
         <v>27</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="G47" s="14" t="s">
         <v>87</v>
+      </c>
+      <c r="H47" s="7" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="30" x14ac:dyDescent="0.25">
@@ -2649,165 +2612,183 @@
         <v>27</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="G48" s="15" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="49" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B49" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="G48" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="49" spans="1:20" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A49" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="D49" s="9"/>
+      <c r="E49" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>150</v>
       </c>
       <c r="G49" s="14" t="s">
         <v>87</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="50" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A50" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G50" s="14" t="s">
-        <v>87</v>
+        <v>157</v>
+      </c>
+    </row>
+    <row r="50" spans="1:20" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A50" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D50" s="5"/>
+      <c r="E50" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="G50" s="13" t="s">
+        <v>128</v>
       </c>
       <c r="H50" s="7" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="51" spans="1:20" ht="30" x14ac:dyDescent="0.25">
-      <c r="A51" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E51" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="I50" s="7"/>
+      <c r="J50" s="7"/>
+      <c r="K50" s="7"/>
+      <c r="L50" s="7"/>
+      <c r="M50" s="7"/>
+      <c r="N50" s="7"/>
+      <c r="O50" s="7"/>
+      <c r="P50" s="7"/>
+      <c r="Q50" s="7"/>
+      <c r="R50" s="7"/>
+      <c r="S50" s="7"/>
+      <c r="T50" s="7"/>
+    </row>
+    <row r="51" spans="1:20" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A51" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C51" s="4"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="G51" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="H51" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="I51" s="7"/>
+      <c r="J51" s="7"/>
+      <c r="K51" s="7"/>
+      <c r="L51" s="7"/>
+      <c r="M51" s="7"/>
+      <c r="N51" s="7"/>
+      <c r="O51" s="7"/>
+      <c r="P51" s="7"/>
+      <c r="Q51" s="7"/>
+      <c r="R51" s="7"/>
+      <c r="S51" s="7"/>
+      <c r="T51" s="7"/>
+    </row>
+    <row r="52" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>48</v>
+      </c>
+      <c r="B52" t="s">
         <v>91</v>
       </c>
-      <c r="F51" s="6" t="s">
+      <c r="C52" t="s">
+        <v>151</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="E52" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="F52" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="G51" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="52" spans="1:20" s="7" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A52" s="10" t="s">
+      <c r="G52" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>48</v>
       </c>
-      <c r="B52" s="10" t="s">
+      <c r="B53" t="s">
         <v>91</v>
       </c>
-      <c r="C52" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="D52" s="9"/>
-      <c r="E52" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="F52" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="G52" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="H52" s="7" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="53" spans="1:20" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A53" s="7" t="s">
+      <c r="C53" t="s">
+        <v>152</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="F53" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="G53" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="54" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>48</v>
       </c>
-      <c r="B53" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="D53" s="5"/>
-      <c r="E53" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F53" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="G53" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="H53" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="I53" s="7"/>
-      <c r="J53" s="7"/>
-      <c r="K53" s="7"/>
-      <c r="L53" s="7"/>
-      <c r="M53" s="7"/>
-      <c r="N53" s="7"/>
-      <c r="O53" s="7"/>
-      <c r="P53" s="7"/>
-      <c r="Q53" s="7"/>
-      <c r="R53" s="7"/>
-      <c r="S53" s="7"/>
-      <c r="T53" s="7"/>
-    </row>
-    <row r="54" spans="1:20" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A54" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B54" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C54" s="4"/>
-      <c r="D54" s="5"/>
+      <c r="B54" t="s">
+        <v>91</v>
+      </c>
+      <c r="C54" t="s">
+        <v>153</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>130</v>
+      </c>
       <c r="E54" s="7" t="s">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="F54" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="G54" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="H54" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="I54" s="7"/>
-      <c r="J54" s="7"/>
-      <c r="K54" s="7"/>
-      <c r="L54" s="7"/>
-      <c r="M54" s="7"/>
-      <c r="N54" s="7"/>
-      <c r="O54" s="7"/>
-      <c r="P54" s="7"/>
-      <c r="Q54" s="7"/>
-      <c r="R54" s="7"/>
-      <c r="S54" s="7"/>
-      <c r="T54" s="7"/>
+        <v>115</v>
+      </c>
+      <c r="G54" s="14" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="55" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
@@ -2817,7 +2798,7 @@
         <v>91</v>
       </c>
       <c r="C55" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D55" s="7" t="s">
         <v>130</v>
@@ -2840,7 +2821,7 @@
         <v>91</v>
       </c>
       <c r="C56" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D56" s="7" t="s">
         <v>130</v>
@@ -2855,144 +2836,145 @@
         <v>87</v>
       </c>
     </row>
-    <row r="57" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+    <row r="57" spans="1:20" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A57" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="G57" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7"/>
+      <c r="J57" s="7"/>
+      <c r="K57" s="7"/>
+      <c r="L57" s="7"/>
+      <c r="M57" s="7"/>
+      <c r="N57" s="7"/>
+      <c r="O57" s="7"/>
+      <c r="P57" s="7"/>
+      <c r="Q57" s="7"/>
+      <c r="R57" s="7"/>
+      <c r="S57" s="7"/>
+      <c r="T57" s="7"/>
+    </row>
+    <row r="58" spans="1:20" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A58" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C58" s="7"/>
+      <c r="D58" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E58" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="F58" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G58" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="H58" s="7"/>
+      <c r="I58" s="7"/>
+      <c r="J58" s="7"/>
+      <c r="K58" s="7"/>
+      <c r="L58" s="7"/>
+      <c r="M58" s="7"/>
+      <c r="N58" s="7"/>
+      <c r="O58" s="7"/>
+      <c r="P58" s="7"/>
+      <c r="Q58" s="7"/>
+      <c r="R58" s="7"/>
+      <c r="S58" s="7"/>
+      <c r="T58" s="7"/>
+    </row>
+    <row r="59" spans="1:20" ht="45.75" x14ac:dyDescent="0.25">
+      <c r="A59" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E59" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C57" t="s">
-        <v>153</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="E57" s="7" t="s">
+      <c r="F59" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="G59" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="H59" s="7"/>
+    </row>
+    <row r="60" spans="1:20" ht="34.5" x14ac:dyDescent="0.25">
+      <c r="A60" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E60" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="F57" s="7" t="s">
+      <c r="F60" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="G57" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="58" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>48</v>
-      </c>
-      <c r="B58" t="s">
-        <v>91</v>
-      </c>
-      <c r="C58" t="s">
-        <v>154</v>
-      </c>
-      <c r="D58" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="E58" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="F58" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="G58" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="59" spans="1:20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>48</v>
-      </c>
-      <c r="B59" t="s">
-        <v>91</v>
-      </c>
-      <c r="C59" t="s">
-        <v>155</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="E59" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="F59" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="G59" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="60" spans="1:20" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A60" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B60" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C60" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D60" s="7"/>
-      <c r="E60" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="F60" s="7" t="s">
-        <v>126</v>
-      </c>
       <c r="G60" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="H60" s="7"/>
-      <c r="I60" s="7"/>
-      <c r="J60" s="7"/>
-      <c r="K60" s="7"/>
-      <c r="L60" s="7"/>
-      <c r="M60" s="7"/>
-      <c r="N60" s="7"/>
-      <c r="O60" s="7"/>
-      <c r="P60" s="7"/>
-      <c r="Q60" s="7"/>
-      <c r="R60" s="7"/>
-      <c r="S60" s="7"/>
-      <c r="T60" s="7"/>
-    </row>
-    <row r="61" spans="1:20" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A61" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B61" s="7" t="s">
+    </row>
+    <row r="61" spans="1:20" ht="34.5" x14ac:dyDescent="0.25">
+      <c r="A61" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E61" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C61" s="7"/>
-      <c r="D61" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="E61" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F61" s="7" t="s">
+      <c r="F61" s="1" t="s">
         <v>39</v>
       </c>
       <c r="G61" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="H61" s="7"/>
-      <c r="I61" s="7"/>
-      <c r="J61" s="7"/>
-      <c r="K61" s="7"/>
-      <c r="L61" s="7"/>
-      <c r="M61" s="7"/>
-      <c r="N61" s="7"/>
-      <c r="O61" s="7"/>
-      <c r="P61" s="7"/>
-      <c r="Q61" s="7"/>
-      <c r="R61" s="7"/>
-      <c r="S61" s="7"/>
-      <c r="T61" s="7"/>
-    </row>
-    <row r="62" spans="1:20" ht="45.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:20" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>50</v>
       </c>
@@ -3000,10 +2982,10 @@
         <v>51</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>91</v>
@@ -3014,7 +2996,6 @@
       <c r="G62" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="H62" s="7"/>
     </row>
     <row r="63" spans="1:20" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
@@ -3024,10 +3005,10 @@
         <v>51</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>91</v>
@@ -3039,7 +3020,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="64" spans="1:20" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:20" ht="165" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>50</v>
       </c>
@@ -3047,19 +3028,22 @@
         <v>51</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="E64" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G64" s="14" t="s">
-        <v>87</v>
+        <v>101</v>
+      </c>
+      <c r="E64" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F64" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="G64" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="H64" s="7" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
@@ -3070,15 +3054,15 @@
         <v>51</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E65" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E65" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="F65" s="6" t="s">
+      <c r="F65" s="7" t="s">
         <v>115</v>
       </c>
       <c r="G65" s="14" t="s">
@@ -3093,22 +3077,22 @@
         <v>51</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="E66" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="E66" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="F66" s="6" t="s">
+      <c r="F66" s="7" t="s">
         <v>115</v>
       </c>
       <c r="G66" s="14" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="165" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>50</v>
       </c>
@@ -3116,25 +3100,22 @@
         <v>51</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="G67" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="H67" s="7" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+      <c r="G67" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>50</v>
       </c>
@@ -3142,19 +3123,22 @@
         <v>51</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E68" s="7" t="s">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="F68" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="G68" s="14" t="s">
-        <v>87</v>
+        <v>161</v>
+      </c>
+      <c r="G68" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="H68" s="7" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
@@ -3165,22 +3149,22 @@
         <v>51</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="E69" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E69" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="F69" s="7" t="s">
+      <c r="F69" s="6" t="s">
         <v>115</v>
       </c>
       <c r="G69" s="14" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>50</v>
       </c>
@@ -3188,22 +3172,22 @@
         <v>51</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E70" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="F70" s="7" t="s">
-        <v>126</v>
+        <v>106</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>115</v>
       </c>
       <c r="G70" s="14" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>50</v>
       </c>
@@ -3211,22 +3195,19 @@
         <v>51</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="E71" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F71" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="G71" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="H71" s="7" t="s">
-        <v>147</v>
+        <v>107</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="G71" s="14" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
@@ -3237,10 +3218,10 @@
         <v>51</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>91</v>
@@ -3260,10 +3241,10 @@
         <v>51</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E73" s="6" t="s">
         <v>91</v>
@@ -3283,22 +3264,16 @@
         <v>51</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E74" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="F74" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="G74" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="75" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+      <c r="G74" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>50</v>
       </c>
@@ -3306,10 +3281,10 @@
         <v>51</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E75" s="6" t="s">
         <v>91</v>
@@ -3321,7 +3296,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" ht="45.75" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>50</v>
       </c>
@@ -3329,22 +3304,25 @@
         <v>51</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E76" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="F76" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="G76" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="77" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="E76" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F76" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="G76" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="H76" s="7" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" ht="57" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>50</v>
       </c>
@@ -3352,16 +3330,22 @@
         <v>51</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="G77" s="15" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="78" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="G77" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>50</v>
       </c>
@@ -3369,10 +3353,10 @@
         <v>51</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>111</v>
+        <v>71</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>113</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>91</v>
@@ -3384,7 +3368,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="45.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>50</v>
       </c>
@@ -3392,22 +3376,13 @@
         <v>51</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="E79" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F79" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="G79" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="H79" s="7" t="s">
-        <v>158</v>
+        <v>72</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="G79" s="15" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="57" x14ac:dyDescent="0.25">
@@ -3418,10 +3393,10 @@
         <v>51</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>112</v>
+        <v>73</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>116</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>91</v>
@@ -3441,10 +3416,10 @@
         <v>51</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E81" s="6" t="s">
         <v>91</v>
@@ -3456,7 +3431,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>50</v>
       </c>
@@ -3464,16 +3439,25 @@
         <v>51</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="D82" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="G82" s="15" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="83" spans="1:8" ht="57" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E82" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="F82" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="G82" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="H82" s="7" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
         <v>50</v>
       </c>
@@ -3481,10 +3465,10 @@
         <v>51</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>91</v>
@@ -3504,10 +3488,10 @@
         <v>51</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>91</v>
@@ -3519,7 +3503,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="85" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
         <v>50</v>
       </c>
@@ -3527,10 +3511,10 @@
         <v>51</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>95</v>
+        <v>78</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>120</v>
       </c>
       <c r="E85" s="7" t="s">
         <v>92</v>
@@ -3540,9 +3524,6 @@
       </c>
       <c r="G85" s="14" t="s">
         <v>87</v>
-      </c>
-      <c r="H85" s="7" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="86" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
@@ -3553,22 +3534,18 @@
         <v>51</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="E86" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="F86" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="G86" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="87" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+      <c r="E86" s="7"/>
+      <c r="F86" s="7"/>
+      <c r="G86" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
         <v>50</v>
       </c>
@@ -3576,22 +3553,16 @@
         <v>51</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="D87" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E87" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="F87" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="G87" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="88" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+      <c r="D87" s="3"/>
+      <c r="E87" s="7"/>
+      <c r="F87" s="7"/>
+      <c r="G87" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
         <v>50</v>
       </c>
@@ -3599,22 +3570,16 @@
         <v>51</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="D88" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="E88" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="F88" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="G88" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="89" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+        <v>176</v>
+      </c>
+      <c r="D88" s="3"/>
+      <c r="E88" s="7"/>
+      <c r="F88" s="7"/>
+      <c r="G88" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
         <v>50</v>
       </c>
@@ -3622,11 +3587,9 @@
         <v>51</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="D89" s="3" t="s">
-        <v>122</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="D89" s="3"/>
       <c r="E89" s="7"/>
       <c r="F89" s="7"/>
       <c r="G89" s="15" t="s">
@@ -3641,7 +3604,7 @@
         <v>51</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D90" s="3"/>
       <c r="E90" s="7"/>
@@ -3650,7 +3613,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
         <v>50</v>
       </c>
@@ -3658,16 +3621,22 @@
         <v>51</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="D91" s="3"/>
-      <c r="E91" s="7"/>
-      <c r="F91" s="7"/>
-      <c r="G91" s="15" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E91" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="F91" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="G91" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A92" s="6" t="s">
         <v>50</v>
       </c>
@@ -3675,16 +3644,16 @@
         <v>51</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="D92" s="3"/>
-      <c r="E92" s="7"/>
-      <c r="F92" s="7"/>
+        <v>81</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>123</v>
+      </c>
       <c r="G92" s="15" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" ht="45.75" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
         <v>50</v>
       </c>
@@ -3692,13 +3661,19 @@
         <v>51</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D93" s="3"/>
-      <c r="E93" s="7"/>
-      <c r="F93" s="7"/>
-      <c r="G93" s="15" t="s">
-        <v>23</v>
+        <v>82</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F93" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="G93" s="14" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
@@ -3709,22 +3684,16 @@
         <v>51</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>80</v>
+        <v>142</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E94" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="F94" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="G94" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="95" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+      <c r="G94" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
         <v>50</v>
       </c>
@@ -3732,16 +3701,14 @@
         <v>51</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="D95" s="3" t="s">
-        <v>123</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="D95" s="3"/>
       <c r="G95" s="15" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="45.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
         <v>50</v>
       </c>
@@ -3749,10 +3716,10 @@
         <v>51</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>91</v>
@@ -3764,178 +3731,192 @@
         <v>87</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A97" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B97" s="6" t="s">
+    <row r="97" spans="1:8" s="7" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A97" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B97" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C97" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="D97" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="G97" s="15" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A98" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B98" s="6" t="s">
+      <c r="C97" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D97" s="5"/>
+      <c r="E97" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F97" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="G97" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="H97" s="7" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" s="7" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A98" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="B98" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C98" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="D98" s="3"/>
-      <c r="G98" s="15" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="99" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+      <c r="C98" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D98" s="5"/>
+      <c r="E98" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F98" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="G98" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="H98" s="7" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" s="6" t="s">
-        <v>50</v>
+        <v>164</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D99" s="3" t="s">
-        <v>125</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="D99" s="6"/>
       <c r="E99" s="6" t="s">
-        <v>91</v>
+        <v>5</v>
       </c>
       <c r="F99" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="G99" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="100" spans="1:8" s="7" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A100" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G99" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="H99" s="6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A100" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E100" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F100" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G100" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A101" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="C101" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="D101" s="2"/>
+      <c r="E101" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F101" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G101" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="H101" s="7"/>
+    </row>
+    <row r="102" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A102" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E102" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="F102" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="G102" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A103" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B103" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E103" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="F103" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="G103" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A104" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="B100" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="C100" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="D100" s="5"/>
-      <c r="E100" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F100" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="G100" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="H100" s="7" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="101" spans="1:8" s="7" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A101" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="B101" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="C101" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="D101" s="5"/>
-      <c r="E101" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F101" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="G101" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="H101" s="7" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A102" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="B102" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C102" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D102" s="6"/>
-      <c r="E102" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F102" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="G102" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="H102" s="6" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="103" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A103" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="B103" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="C103" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="E103" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="F103" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="G103" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="104" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A104" s="6" t="s">
-        <v>175</v>
-      </c>
       <c r="B104" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="C104" s="17" t="s">
-        <v>178</v>
-      </c>
-      <c r="D104" s="2"/>
+        <v>184</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>183</v>
+      </c>
       <c r="E104" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="F104" s="6" t="s">
-        <v>177</v>
+        <v>181</v>
+      </c>
+      <c r="F104" s="7" t="s">
+        <v>182</v>
       </c>
       <c r="G104" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="H104" s="7"/>
     </row>
     <row r="105" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
-        <v>4</v>
+        <v>175</v>
       </c>
       <c r="B105" s="6" t="s">
         <v>184</v>
@@ -3958,7 +3939,7 @@
     </row>
     <row r="106" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A106" s="7" t="s">
-        <v>21</v>
+        <v>171</v>
       </c>
       <c r="B106" s="6" t="s">
         <v>184</v>
@@ -3979,77 +3960,8 @@
         <v>87</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A107" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="B107" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="C107" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="D107" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="E107" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="F107" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="G107" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="108" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A108" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="B108" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="C108" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="D108" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="E108" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="F108" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="G108" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="109" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A109" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="B109" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="C109" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="D109" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="E109" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="F109" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="G109" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:A103" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:A100" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
@@ -4057,15 +3969,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100919AB8A12910594B8F4D80F4ACA7D0E7" ma:contentTypeVersion="6" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9c71394a73500791d9f4b659570ff6f6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a318c9bd-5828-4914-8ac9-a57d8c01df7a" xmlns:ns3="4da7f078-0f32-436f-b12a-21525bae5a0e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f0993cb8e7f28d1e7915cb051b812a71" ns2:_="" ns3:_="">
     <xsd:import namespace="a318c9bd-5828-4914-8ac9-a57d8c01df7a"/>
@@ -4242,6 +4145,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -4249,14 +4161,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B8261F5-E2C2-49F8-99F3-13EB69507EB7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56F0D49C-4924-48A7-977F-FB48DDC11B03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4275,6 +4179,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B8261F5-E2C2-49F8-99F3-13EB69507EB7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC4DE233-B05C-40D4-9E0D-B697BD35B3E3}">
   <ds:schemaRefs>

</xml_diff>